<commit_message>
Publish Halifax_2009_WCH, Szeged_2010_WC, Poznan_2009_WC, Poznan_2010_WCH, Szeged_2011_WCH, Szeged_2009_WC, Vichy_2010_WC, Duisburg_2010_WC, Banyoles_2010_MAR, Moscow_2009_JWCH, Racice_2009_WC, Crestuma_2009_MAR, Poznan_2012_WC, Rome_2012_MAR
</commit_message>
<xml_diff>
--- a/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
+++ b/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
@@ -4170,11 +4170,6 @@
           <t>0:00:47.090</t>
         </is>
       </c>
-      <c r="R57" t="inlineStr">
-        <is>
-          <t>100316</t>
-        </is>
-      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -10561,11 +10556,6 @@
           <t>0:07:39.330</t>
         </is>
       </c>
-      <c r="S154" t="inlineStr">
-        <is>
-          <t>85433</t>
-        </is>
-      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12739,16 +12729,6 @@
           <t>0:02:34.860</t>
         </is>
       </c>
-      <c r="R187" t="inlineStr">
-        <is>
-          <t>90936</t>
-        </is>
-      </c>
-      <c r="S187" t="inlineStr">
-        <is>
-          <t>168691</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -15237,11 +15217,6 @@
           <t>2:13:48.032</t>
         </is>
       </c>
-      <c r="R226" t="inlineStr">
-        <is>
-          <t>119523</t>
-        </is>
-      </c>
     </row>
     <row r="227">
       <c r="A227" t="inlineStr">
@@ -15304,11 +15279,6 @@
       <c r="Q227" t="inlineStr">
         <is>
           <t>0:00:01.998</t>
-        </is>
-      </c>
-      <c r="R227" t="inlineStr">
-        <is>
-          <t>146367</t>
         </is>
       </c>
     </row>
@@ -21116,7 +21086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D144"/>
+  <dimension ref="A1:D138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -21760,61 +21730,61 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>119523</t>
+          <t>35984</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Ben</t>
+          <t>Agnes</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BROWN</t>
+          <t>BRUN-LIE</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>35984</t>
+          <t>42728</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Agnes</t>
+          <t>Juan Ignacio</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>BRUN-LIE</t>
+          <t>CACERES</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>146367</t>
+          <t>72465</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Raul</t>
+          <t>Enrico Paolo Guido</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>FERNANDEZ BUSTO</t>
+          <t>CALVI</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -21826,17 +21796,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>42728</t>
+          <t>46822</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Juan Ignacio</t>
+          <t>Manuel Antonio</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CACERES</t>
+          <t>CAMPOS</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -21848,17 +21818,17 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>72465</t>
+          <t>42428</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Enrico Paolo Guido</t>
+          <t>Riccardo</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CALVI</t>
+          <t>CECCHINI</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -21870,17 +21840,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>46822</t>
+          <t>146571</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Manuel Antonio</t>
+          <t>David</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CAMPOS</t>
+          <t>CEDDIA</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -21892,17 +21862,17 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>42428</t>
+          <t>45212</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Riccardo</t>
+          <t>Benjamin</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>CECCHINI</t>
+          <t>CEINER</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -21914,105 +21884,105 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>146571</t>
+          <t>50186</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>David</t>
+          <t>Stefania</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CEDDIA</t>
+          <t>CICALI</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>45212</t>
+          <t>36581</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Benjamin</t>
+          <t>Susanna</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>CEINER</t>
+          <t>CICALI</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>50186</t>
+          <t>42535</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Stefania</t>
+          <t>Remi</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>CICALI</t>
+          <t>CLIN</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>36581</t>
+          <t>53066</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Susanna</t>
+          <t>Stanton</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CICALI</t>
+          <t>COLLINS</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>42535</t>
+          <t>83363</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Remi</t>
+          <t>Albert</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>CLIN</t>
+          <t>COROMINAS BERTRAN</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -22024,17 +21994,17 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>53066</t>
+          <t>48801</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Stanton</t>
+          <t>Tom</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>COLLINS</t>
+          <t>CREMERS</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -22046,39 +22016,39 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>83363</t>
+          <t>47431</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Albert</t>
+          <t>Renata</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>COROMINAS BERTRAN</t>
+          <t>CSAY</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>48801</t>
+          <t>36231</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Tom</t>
+          <t>Andrew</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>CREMERS</t>
+          <t>DANIELS</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -22090,39 +22060,39 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>47431</t>
+          <t>86064</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Renata</t>
+          <t>Juliano</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>CSAY</t>
+          <t>DARLAN CRAI DAL MOLIN</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>36231</t>
+          <t>36604</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Andrew</t>
+          <t>Miika</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>DANIELS</t>
+          <t>DIETRICH</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -22134,17 +22104,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>86064</t>
+          <t>63503</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Juliano</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>DARLAN CRAI DAL MOLIN</t>
+          <t>DLOUHY</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -22156,17 +22126,17 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>36604</t>
+          <t>118913</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Miika</t>
+          <t>Vojtech</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>DIETRICH</t>
+          <t>DLOUHY</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -22178,17 +22148,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>63503</t>
+          <t>54196</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Victor</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>DLOUHY</t>
+          <t>DOUX</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -22200,17 +22170,17 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>118913</t>
+          <t>46679</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Vojtech</t>
+          <t>Vaclav</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>DLOUHY</t>
+          <t>DUBSKY</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -22222,17 +22192,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>54196</t>
+          <t>49670</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Victor</t>
+          <t>Adam</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>DOUX</t>
+          <t>DOCZE</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -22244,17 +22214,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>46679</t>
+          <t>49755</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Vaclav</t>
+          <t>Matthias</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>DUBSKY</t>
+          <t>EBHARDT</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
@@ -22266,39 +22236,39 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>49670</t>
+          <t>42797</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Adam</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>DOCZE</t>
+          <t>EGAN-SIMMONS</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>49755</t>
+          <t>42798</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Matthias</t>
+          <t>Peter</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EBHARDT</t>
+          <t>EGAN</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
@@ -22310,17 +22280,17 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>42797</t>
+          <t>42425</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Agata</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>EGAN-SIMMONS</t>
+          <t>FANTINI</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
@@ -22332,17 +22302,17 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>42798</t>
+          <t>49433</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Peter</t>
+          <t>Alvaro</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>EGAN</t>
+          <t>FERNANDEZ FIUZA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
@@ -22354,17 +22324,17 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>42425</t>
+          <t>46840</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Agata</t>
+          <t>Tania</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>FANTINI</t>
+          <t>FERNANDEZ</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
@@ -22376,17 +22346,17 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>49433</t>
+          <t>50159</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Alvaro</t>
+          <t>Luca</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>FERNANDEZ FIUZA</t>
+          <t>FERRAINA</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
@@ -22398,61 +22368,61 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>46840</t>
+          <t>49518</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Tania</t>
+          <t>Ramon</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>FERNANDEZ</t>
+          <t>FERRO</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>50159</t>
+          <t>63447</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Luca</t>
+          <t>Tegan</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>FERRAINA</t>
+          <t>FRASER</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>49518</t>
+          <t>63242</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Ramon</t>
+          <t>Manuel</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FERRO</t>
+          <t>GARRIDO</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -22464,17 +22434,17 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>63447</t>
+          <t>64651</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Tegan</t>
+          <t>Francesca</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>FRASER</t>
+          <t>GENZO</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
@@ -22486,17 +22456,17 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>63242</t>
+          <t>61538</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Manuel</t>
+          <t>Alessandro</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>GARRIDO</t>
+          <t>GNECCHI</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
@@ -22508,39 +22478,39 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>64651</t>
+          <t>50155</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Francesca</t>
+          <t>Matteo</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>GENZO</t>
+          <t>GRAZIANI</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>61538</t>
+          <t>49668</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Alessandro</t>
+          <t>Attila</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>GNECCHI</t>
+          <t>GYORE</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
@@ -22552,39 +22522,39 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>168691</t>
+          <t>36391</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Martin</t>
+          <t>Bridgitte</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>GONZALEZ FERNANDEZ</t>
+          <t>HARTLEY</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>50155</t>
+          <t>48492</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Matteo</t>
+          <t>Albert</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>GRAZIANI</t>
+          <t>HICKS</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
@@ -22596,17 +22566,17 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>49668</t>
+          <t>35993</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Attila</t>
+          <t>Lars</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>GYORE</t>
+          <t>HJEMDAL</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
@@ -22618,17 +22588,17 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>36391</t>
+          <t>45228</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Bridgitte</t>
+          <t>Noemi</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>HARTLEY</t>
+          <t>HORVATH</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
@@ -22640,17 +22610,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>100316</t>
+          <t>46372</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Miguel</t>
+          <t>Dmytro</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>ERGUETA RODRIGUEZ</t>
+          <t>IANCHUK</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -22662,105 +22632,105 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>48492</t>
+          <t>48496</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Albert</t>
+          <t>Jenny</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>HICKS</t>
+          <t>ILLIDGE</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>35993</t>
+          <t>48954</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Lars</t>
+          <t>Tanja</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>HJEMDAL</t>
+          <t>JANTUNEN</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>45228</t>
+          <t>49732</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Noemi</t>
+          <t>Tomas</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>HORVATH</t>
+          <t>JEZEK</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>46372</t>
+          <t>47633</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Dmytro</t>
+          <t>Karin</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>IANCHUK</t>
+          <t>JOHANSSON</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>48496</t>
+          <t>49753</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Jenny</t>
+          <t>Michaela</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>ILLIDGE</t>
+          <t>LINDBLAD JONSSON</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
@@ -22772,39 +22742,39 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>48954</t>
+          <t>42270</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Tanja</t>
+          <t>Mateusz</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>JANTUNEN</t>
+          <t>KAMINSKI</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>49732</t>
+          <t>140359</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Tomas</t>
+          <t>Brendan</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>JEZEK</t>
+          <t>KEYS</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
@@ -22816,17 +22786,17 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>47633</t>
+          <t>49657</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Karin</t>
+          <t>Vanda</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>JOHANSSON</t>
+          <t>KISZLI</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
@@ -22838,17 +22808,17 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>49753</t>
+          <t>64839</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Michaela</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>LINDBLAD JONSSON</t>
+          <t>KLEIN</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
@@ -22860,17 +22830,17 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>42270</t>
+          <t>45220</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Mateusz</t>
+          <t>David Gyorgy</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>KAMINSKI</t>
+          <t>KORISANSZKY</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -22882,17 +22852,17 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>140359</t>
+          <t>35937</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Brendan</t>
+          <t>Arkadiusz</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>KEYS</t>
+          <t>KRAJEWSKI</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
@@ -22904,61 +22874,61 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>49657</t>
+          <t>49666</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Vanda</t>
+          <t>Marton</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>KISZLI</t>
+          <t>KOVER</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>64839</t>
+          <t>48163</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Rui</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>KLEIN</t>
+          <t>LACERDA</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>45220</t>
+          <t>49267</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>David Gyorgy</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>KORISANSZKY</t>
+          <t>LEVERETT</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
@@ -22970,17 +22940,17 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>35937</t>
+          <t>52099</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Arkadiusz</t>
+          <t>Joakim</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>KRAJEWSKI</t>
+          <t>LINDBERG</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
@@ -22992,17 +22962,17 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>49666</t>
+          <t>42771</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Marton</t>
+          <t>Nikica</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>KOVER</t>
+          <t>LJUBEK</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
@@ -23014,17 +22984,17 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>48163</t>
+          <t>35385</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Rui</t>
+          <t>Edwin</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>LACERDA</t>
+          <t>LUCAS</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
@@ -23036,17 +23006,17 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>49267</t>
+          <t>42364</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Jan</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
         <is>
-          <t>LEVERETT</t>
+          <t>LUNACEK</t>
         </is>
       </c>
       <c r="D88" t="inlineStr">
@@ -23058,17 +23028,17 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>52099</t>
+          <t>42660</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Joakim</t>
+          <t>Pierrick</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>LINDBERG</t>
+          <t>MARTIN</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
@@ -23080,39 +23050,39 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>42771</t>
+          <t>52179</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Nikica</t>
+          <t>Catherine</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>LJUBEK</t>
+          <t>MCARTHUR</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>35385</t>
+          <t>48221</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Edwin</t>
+          <t>Sean</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>LUCAS</t>
+          <t>MCCARTHY</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
@@ -23124,39 +23094,39 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>42364</t>
+          <t>42361</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Jan</t>
+          <t>Kaitlyn</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>LUNACEK</t>
+          <t>MCELROY</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>42660</t>
+          <t>35992</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Pierrick</t>
+          <t>Morten</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>MARTIN</t>
+          <t>MINDE</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
@@ -23168,17 +23138,17 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>52179</t>
+          <t>35393</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Catherine</t>
+          <t>Gwendoline</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MCARTHUR</t>
+          <t>MOREL</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
@@ -23190,61 +23160,61 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>48221</t>
+          <t>42427</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Sean</t>
+          <t>Federica</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>MCCARTHY</t>
+          <t>NOLE</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>42361</t>
+          <t>49662</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Kaitlyn</t>
+          <t>Balint</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>MCELROY</t>
+          <t>NOE</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>85433</t>
+          <t>42369</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Ruben</t>
+          <t>Michael</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>RODRIGUEZ GIL</t>
+          <t>ODVARKO</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
@@ -23256,17 +23226,17 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>35992</t>
+          <t>68942</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Morten</t>
+          <t>Radoslav</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>MINDE</t>
+          <t>OLSZEWSKI</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
@@ -23278,39 +23248,39 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>90936</t>
+          <t>49441</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Amaia</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>ALVAREZ LLANO</t>
+          <t>OSABA OLABERRI</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>35393</t>
+          <t>51871</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Gwendoline</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>MOREL</t>
+          <t>PALDANIUS</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
@@ -23322,83 +23292,83 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>42427</t>
+          <t>41784</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Federica</t>
+          <t>Laurens</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>NOLE</t>
+          <t>PANNECOUCKE</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>49662</t>
+          <t>46832</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Balint</t>
+          <t>Laura</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>NOE</t>
+          <t>PEDRUELO</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>42369</t>
+          <t>41793</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Michael</t>
+          <t>Hermien</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>ODVARKO</t>
+          <t>PETERS</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>68942</t>
+          <t>41787</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Radoslav</t>
+          <t>William</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>OLSZEWSKI</t>
+          <t>PETERS</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
@@ -23410,17 +23380,17 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>49441</t>
+          <t>50157</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Amaia</t>
+          <t>Gaia</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>OSABA OLABERRI</t>
+          <t>PIAZZA</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
@@ -23432,39 +23402,39 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>51871</t>
+          <t>49620</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Sofia</t>
+          <t>Orion</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>PALDANIUS</t>
+          <t>PILO</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>41784</t>
+          <t>36448</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Laurens</t>
+          <t>Fernando</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>PANNECOUCKE</t>
+          <t>PIMENTA</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
@@ -23476,61 +23446,61 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>46832</t>
+          <t>53954</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Laura</t>
+          <t>Bartosz</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>PEDRUELO</t>
+          <t>PLAWSKI</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>41793</t>
+          <t>175192</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Hermien</t>
+          <t>Luis</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>PETERS</t>
+          <t>BLANCO COBIAN</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>41787</t>
+          <t>48161</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>William</t>
+          <t>Jose</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>PETERS</t>
+          <t>RAMALHO</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
@@ -23542,39 +23512,39 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>50157</t>
+          <t>49767</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Gaia</t>
+          <t>Felix</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>PIAZZA</t>
+          <t>RICHTER</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>49620</t>
+          <t>36568</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Orion</t>
+          <t>Nicola</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>PILO</t>
+          <t>RIPAMONTI</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
@@ -23586,17 +23556,17 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>36448</t>
+          <t>46825</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Fernando</t>
+          <t>Diego</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>PIMENTA</t>
+          <t>ROMERO</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
@@ -23608,17 +23578,17 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>53954</t>
+          <t>35981</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Bartosz</t>
+          <t>Daniel</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>PLAWSKI</t>
+          <t>SALBU</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
@@ -23630,17 +23600,17 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>175192</t>
+          <t>57974</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Luis</t>
+          <t>Alejandro</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>BLANCO COBIAN</t>
+          <t>SANCHEZ COBOS</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
@@ -23652,39 +23622,39 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>48161</t>
+          <t>48740</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Jose</t>
+          <t>Kerry</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>RAMALHO</t>
+          <t>SEGAL</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>49767</t>
+          <t>46397</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Felix</t>
+          <t>Eduard</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>RICHTER</t>
+          <t>SHEMETYLO</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
@@ -23696,17 +23666,17 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>36568</t>
+          <t>36449</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Nicola</t>
+          <t>Emanuel</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>RIPAMONTI</t>
+          <t>SILVA</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
@@ -23718,17 +23688,17 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>46825</t>
+          <t>105917</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Diego</t>
+          <t>Jakub</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>ROMERO</t>
+          <t>SITKOWSKI</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
@@ -23740,17 +23710,17 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>35981</t>
+          <t>35869</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Daniel</t>
+          <t>Vincent</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>SALBU</t>
+          <t>SLOMINSKI</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
@@ -23762,17 +23732,17 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>57974</t>
+          <t>35980</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Alejandro</t>
+          <t>Jo Sondre</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>SANCHEZ COBOS</t>
+          <t>SOLHAUG</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
@@ -23784,39 +23754,39 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>48740</t>
+          <t>49664</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>Kerry</t>
+          <t>Laszlo</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>SEGAL</t>
+          <t>SOLTI</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>46397</t>
+          <t>97457</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>Eduard</t>
+          <t>Branislav</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>SHEMETYLO</t>
+          <t>SRAMEK</t>
         </is>
       </c>
       <c r="D123" t="inlineStr">
@@ -23828,61 +23798,61 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>36449</t>
+          <t>47622</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>Emanuel</t>
+          <t>Linnea</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>SILVA</t>
+          <t>STENSILS</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>105917</t>
+          <t>84966</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
         <is>
-          <t>Jakub</t>
+          <t>Jennifer</t>
         </is>
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SITKOWSKI</t>
+          <t>STEVENS</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>M</t>
+          <t>F</t>
         </is>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>35869</t>
+          <t>53100</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>Vincent</t>
+          <t>Kristof Zoltan</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>SLOMINSKI</t>
+          <t>SZABO</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
@@ -23894,17 +23864,17 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>35980</t>
+          <t>52576</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
         <is>
-          <t>Jo Sondre</t>
+          <t>Guang Yi Lucas</t>
         </is>
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>SOLHAUG</t>
+          <t>TEO</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
@@ -23916,17 +23886,17 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>49664</t>
+          <t>48841</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>Laszlo</t>
+          <t>Jonathan</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SOLTI</t>
+          <t>TYE</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
@@ -23938,17 +23908,17 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>97457</t>
+          <t>48410</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>Branislav</t>
+          <t>Brandon</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>SRAMEK</t>
+          <t>VAN DER WALT</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
@@ -23960,17 +23930,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>47622</t>
+          <t>73769</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
-          <t>Linnea</t>
+          <t>Melanie</t>
         </is>
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>STENSILS</t>
+          <t>VAN NIEKERK</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
@@ -23982,39 +23952,39 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>84966</t>
+          <t>100226</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
         <is>
-          <t>Jennifer</t>
+          <t>Ernest</t>
         </is>
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>STEVENS</t>
+          <t>VAN RIET</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>M</t>
         </is>
       </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>53100</t>
+          <t>63247</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>Kristof Zoltan</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SZABO</t>
+          <t>VEGA VEGA</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
@@ -24026,17 +23996,17 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>52576</t>
+          <t>36586</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>Guang Yi Lucas</t>
+          <t>Filippo</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>TEO</t>
+          <t>VINCENZI</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
@@ -24048,17 +24018,17 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>48841</t>
+          <t>45222</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
-          <t>Jonathan</t>
+          <t>Viktor</t>
         </is>
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>TYE</t>
+          <t>VIOLA</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
@@ -24070,17 +24040,17 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>48410</t>
+          <t>36743</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>Brandon</t>
+          <t>Eivind</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>VAN DER WALT</t>
+          <t>VOLD</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
@@ -24092,17 +24062,17 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>73769</t>
+          <t>49659</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>Melanie</t>
+          <t>Eniko</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VAN NIEKERK</t>
+          <t>VACZAI</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
@@ -24114,17 +24084,17 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>100226</t>
+          <t>41792</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>Ernest</t>
+          <t>Joeri</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>VAN RIET</t>
+          <t>WECKX</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
@@ -24136,152 +24106,20 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>63247</t>
+          <t>90974</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
         <is>
-          <t>Carlos</t>
+          <t>Patrick</t>
         </is>
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>VEGA VEGA</t>
+          <t>WOELFEL</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="139">
-      <c r="A139" t="inlineStr">
-        <is>
-          <t>36586</t>
-        </is>
-      </c>
-      <c r="B139" t="inlineStr">
-        <is>
-          <t>Filippo</t>
-        </is>
-      </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>VINCENZI</t>
-        </is>
-      </c>
-      <c r="D139" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="140">
-      <c r="A140" t="inlineStr">
-        <is>
-          <t>45222</t>
-        </is>
-      </c>
-      <c r="B140" t="inlineStr">
-        <is>
-          <t>Viktor</t>
-        </is>
-      </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>VIOLA</t>
-        </is>
-      </c>
-      <c r="D140" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="141">
-      <c r="A141" t="inlineStr">
-        <is>
-          <t>36743</t>
-        </is>
-      </c>
-      <c r="B141" t="inlineStr">
-        <is>
-          <t>Eivind</t>
-        </is>
-      </c>
-      <c r="C141" t="inlineStr">
-        <is>
-          <t>VOLD</t>
-        </is>
-      </c>
-      <c r="D141" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="142">
-      <c r="A142" t="inlineStr">
-        <is>
-          <t>49659</t>
-        </is>
-      </c>
-      <c r="B142" t="inlineStr">
-        <is>
-          <t>Eniko</t>
-        </is>
-      </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>VACZAI</t>
-        </is>
-      </c>
-      <c r="D142" t="inlineStr">
-        <is>
-          <t>F</t>
-        </is>
-      </c>
-    </row>
-    <row r="143">
-      <c r="A143" t="inlineStr">
-        <is>
-          <t>41792</t>
-        </is>
-      </c>
-      <c r="B143" t="inlineStr">
-        <is>
-          <t>Joeri</t>
-        </is>
-      </c>
-      <c r="C143" t="inlineStr">
-        <is>
-          <t>WECKX</t>
-        </is>
-      </c>
-      <c r="D143" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="144">
-      <c r="A144" t="inlineStr">
-        <is>
-          <t>90974</t>
-        </is>
-      </c>
-      <c r="B144" t="inlineStr">
-        <is>
-          <t>Patrick</t>
-        </is>
-      </c>
-      <c r="C144" t="inlineStr">
-        <is>
-          <t>WOELFEL</t>
-        </is>
-      </c>
-      <c r="D144" t="inlineStr">
         <is>
           <t>M</t>
         </is>

</xml_diff>

<commit_message>
Publish Halifax_2009_WCH, Duisburg_2011_WC, Szeged_2014_JWCH, Minsk_2016_JWCH, Rome_2012_MAR, Banyoles_2010_MAR, Crestuma_2009_MAR
</commit_message>
<xml_diff>
--- a/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
+++ b/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
@@ -14191,6 +14191,11 @@
           <t>2:07:13.590</t>
         </is>
       </c>
+      <c r="R210" t="inlineStr">
+        <is>
+          <t>58775</t>
+        </is>
+      </c>
     </row>
     <row r="211">
       <c r="A211" t="inlineStr">
@@ -18699,6 +18704,11 @@
           <t>0:03:31.300</t>
         </is>
       </c>
+      <c r="R279" t="inlineStr">
+        <is>
+          <t>58775</t>
+        </is>
+      </c>
     </row>
     <row r="280">
       <c r="A280" t="inlineStr">
@@ -19436,6 +19446,11 @@
       <c r="Q290" t="inlineStr">
         <is>
           <t>0:00:16.120</t>
+        </is>
+      </c>
+      <c r="R290" t="inlineStr">
+        <is>
+          <t>58936</t>
         </is>
       </c>
     </row>
@@ -21086,7 +21101,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D138"/>
+  <dimension ref="A1:D140"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24125,6 +24140,50 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>58775</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>Nuno</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>BARROS</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>58936</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>Nestor</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>PINTA</t>
+        </is>
+      </c>
+      <c r="D140" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Szeged_2024_WC, Halifax_2022_WCH, PonteDeLima_2022_MAR, Szeged_2022_JWCH, Montemor_2021_JWCH, Szeged_2021_WC, Pitesti_2019_JWCH, Szeged_2017_WC, Minsk_2016_JWCH, Copenhagen_2015_WC, Montemor_2015_JWCH, OklahomaCity_2014_MAR, Szeged_2014_JWCH, Copenhagen_2013_MAR, Duisburg_2013_WCH, Racice_2013_WC, Szeged_2013_WC, Welland_2013_JWCH, Duisburg_2012_WC, Moscow_2012_WC, Poznan_2012_WC, Rome_2012_MAR, Duisburg_2011_WC, Szeged_2011_WCH, Banyoles_2010_MAR, Duisburg_2010_WC, Poznan_2010_WCH, Szeged_2010_WC, Vichy_2010_WC, Moscow_2009_JWCH, Poznan_2009_WC, Racice_2009_WC, Szeged_2009_WC
</commit_message>
<xml_diff>
--- a/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
+++ b/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
@@ -10586,6 +10586,11 @@
           <t>0:07:39.330</t>
         </is>
       </c>
+      <c r="S154" t="inlineStr">
+        <is>
+          <t>47619</t>
+        </is>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -12759,6 +12764,11 @@
           <t>0:02:34.860</t>
         </is>
       </c>
+      <c r="S187" t="inlineStr">
+        <is>
+          <t>72616</t>
+        </is>
+      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -15250,6 +15260,11 @@
       <c r="P226" t="inlineStr">
         <is>
           <t>2:13:48.032</t>
+        </is>
+      </c>
+      <c r="R226" t="inlineStr">
+        <is>
+          <t>119523</t>
         </is>
       </c>
     </row>
@@ -21171,7 +21186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D153"/>
+  <dimension ref="A1:D156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24540,6 +24555,72 @@
         </is>
       </c>
     </row>
+    <row r="154">
+      <c r="A154" t="inlineStr">
+        <is>
+          <t>47619</t>
+        </is>
+      </c>
+      <c r="B154" t="inlineStr">
+        <is>
+          <t>Ruben</t>
+        </is>
+      </c>
+      <c r="C154" t="inlineStr">
+        <is>
+          <t>MILLAN</t>
+        </is>
+      </c>
+      <c r="D154" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>72616</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Adrian</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>GONZALEZ</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>119523</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Ben</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>BROWN</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Montemor_2021_JWCH, Belgrade_2017_WC, Szeged_2017_WC, Welland_2013_JWCH, Rome_2012_MAR, Poznan_2012_WC, Szeged_2011_WCH, Duisburg_2011_WC, Banyoles_2010_MAR, Poznan_2010_WCH, Duisburg_2010_WC, Szeged_2010_WC, Vichy_2010_WC, Crestuma_2009_MAR, Halifax_2009_WCH, Szeged_2009_WC, Poznan_2009_WC, Racice_2009_WC
</commit_message>
<xml_diff>
--- a/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
+++ b/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
@@ -12764,11 +12764,6 @@
           <t>0:02:34.860</t>
         </is>
       </c>
-      <c r="S187" t="inlineStr">
-        <is>
-          <t>72616</t>
-        </is>
-      </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
@@ -15260,11 +15255,6 @@
       <c r="P226" t="inlineStr">
         <is>
           <t>2:13:48.032</t>
-        </is>
-      </c>
-      <c r="R226" t="inlineStr">
-        <is>
-          <t>119523</t>
         </is>
       </c>
     </row>
@@ -21186,7 +21176,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D156"/>
+  <dimension ref="A1:D154"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24577,50 +24567,6 @@
         </is>
       </c>
     </row>
-    <row r="155">
-      <c r="A155" t="inlineStr">
-        <is>
-          <t>72616</t>
-        </is>
-      </c>
-      <c r="B155" t="inlineStr">
-        <is>
-          <t>Adrian</t>
-        </is>
-      </c>
-      <c r="C155" t="inlineStr">
-        <is>
-          <t>GONZALEZ</t>
-        </is>
-      </c>
-      <c r="D155" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
-    <row r="156">
-      <c r="A156" t="inlineStr">
-        <is>
-          <t>119523</t>
-        </is>
-      </c>
-      <c r="B156" t="inlineStr">
-        <is>
-          <t>Ben</t>
-        </is>
-      </c>
-      <c r="C156" t="inlineStr">
-        <is>
-          <t>BROWN</t>
-        </is>
-      </c>
-      <c r="D156" t="inlineStr">
-        <is>
-          <t>M</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Publish Banyoles_2010_MAR, Duisburg_2010_WC, Poznan_2010_WCH, Vichy_2010_WC
</commit_message>
<xml_diff>
--- a/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
+++ b/events/Banyoles_2010_MAR/Banyoles_2010_MAR_Results.xlsx
@@ -2261,6 +2261,11 @@
           <t>0:14:21.630</t>
         </is>
       </c>
+      <c r="R27" t="inlineStr">
+        <is>
+          <t>61292</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -4712,6 +4717,11 @@
           <t>0:08:54.570</t>
         </is>
       </c>
+      <c r="R65" t="inlineStr">
+        <is>
+          <t>42510</t>
+        </is>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -11704,6 +11714,11 @@
       <c r="Q171" t="inlineStr">
         <is>
           <t>0:02:12.150</t>
+        </is>
+      </c>
+      <c r="R171" t="inlineStr">
+        <is>
+          <t>49637</t>
         </is>
       </c>
     </row>
@@ -21176,7 +21191,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D154"/>
+  <dimension ref="A1:D157"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -24567,6 +24582,72 @@
         </is>
       </c>
     </row>
+    <row r="155">
+      <c r="A155" t="inlineStr">
+        <is>
+          <t>61292</t>
+        </is>
+      </c>
+      <c r="B155" t="inlineStr">
+        <is>
+          <t>Malin</t>
+        </is>
+      </c>
+      <c r="C155" t="inlineStr">
+        <is>
+          <t>TITOTIC</t>
+        </is>
+      </c>
+      <c r="D155" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="156">
+      <c r="A156" t="inlineStr">
+        <is>
+          <t>42510</t>
+        </is>
+      </c>
+      <c r="B156" t="inlineStr">
+        <is>
+          <t>Yul</t>
+        </is>
+      </c>
+      <c r="C156" t="inlineStr">
+        <is>
+          <t>OELZE</t>
+        </is>
+      </c>
+      <c r="D156" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+    </row>
+    <row r="157">
+      <c r="A157" t="inlineStr">
+        <is>
+          <t>49637</t>
+        </is>
+      </c>
+      <c r="B157" t="inlineStr">
+        <is>
+          <t>Sofie</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
+          <t>JØRGENSEN</t>
+        </is>
+      </c>
+      <c r="D157" t="inlineStr">
+        <is>
+          <t>F</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>